<commit_message>
feat: expose workbook permeability policy
</commit_message>
<xml_diff>
--- a/test_data/examples/smeaheia/smeaheia_workbook.xlsx
+++ b/test_data/examples/smeaheia/smeaheia_workbook.xlsx
@@ -587,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -615,77 +615,77 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>water_depth</t>
+          <t>target_dz_water</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>312</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>reservoir_top</t>
+          <t>target_dz_overburden</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1214.5</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>bottom_depth</t>
+          <t>target_dz_reservoir</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3162.5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>target_dz_water</t>
+          <t>reservoir_permx</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>50</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>target_dz_overburden</t>
+          <t>overburden_permx</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>60</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>target_dz_reservoir</t>
+          <t>cells_per_layer</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10</v>
+        <v>400</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>cells_per_layer</t>
+          <t>min_water_layers</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>400</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>min_water_layers</t>
+          <t>min_overburden_layers</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -695,20 +695,10 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>min_overburden_layers</t>
+          <t>min_reservoir_layers</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>min_reservoir_layers</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Declare and validate WellClass-to-GaP units
</commit_message>
<xml_diff>
--- a/test_data/examples/smeaheia/smeaheia_workbook.xlsx
+++ b/test_data/examples/smeaheia/smeaheia_workbook.xlsx
@@ -587,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -605,100 +605,124 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>top_depth</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>4</v>
+          <t>depth_unit</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>target_dz_water</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>50</v>
+          <t>permeability_unit</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>mD</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>target_dz_overburden</t>
+          <t>top_depth</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>60</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>target_dz_reservoir</t>
+          <t>target_dz_water</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>10</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>reservoir_permx</t>
+          <t>target_dz_overburden</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1000</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>overburden_permx</t>
+          <t>target_dz_reservoir</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.001</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>cells_per_layer</t>
+          <t>reservoir_permx</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>400</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>min_water_layers</t>
+          <t>overburden_permx</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>min_overburden_layers</t>
+          <t>cells_per_layer</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1</v>
+        <v>400</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>min_water_layers</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>min_overburden_layers</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>min_reservoir_layers</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B13" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1482,7 +1506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1526,6 +1550,16 @@
           <t>p_resrv</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>depth_unit</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>pressure_unit</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1556,6 +1590,16 @@
       <c r="H2" t="n">
         <v>129.99</v>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1585,6 +1629,16 @@
       </c>
       <c r="H3" t="n">
         <v>131</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Use mass-fraction salinity across pressure and CIRRUS
</commit_message>
<xml_diff>
--- a/test_data/examples/smeaheia/smeaheia_workbook.xlsx
+++ b/test_data/examples/smeaheia/smeaheia_workbook.xlsx
@@ -1506,7 +1506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1560,6 +1560,16 @@
           <t>pressure_unit</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>salinity_basis</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>salinity</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1600,6 +1610,14 @@
           <t>bar</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>mass_fraction</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>0.032</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1639,6 +1657,14 @@
         <is>
           <t>bar</t>
         </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>mass_fraction</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>0.032</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add DesignMatrix permeability overrides
Introduce the DesignMatrix sheet with backwards-compatible SubsurfaceAssumptions parsing, apply per-scenario grid and well-material permeability overrides, and record effective values for reproducibility.
</commit_message>
<xml_diff>
--- a/test_data/examples/smeaheia/smeaheia_workbook.xlsx
+++ b/test_data/examples/smeaheia/smeaheia_workbook.xlsx
@@ -14,7 +14,7 @@
     <sheet name="HoleCasings" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Plugs" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Stratigraphy" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="SubsurfaceAssumptions" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="DesignMatrix" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Notes" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
@@ -1506,7 +1506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:R3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1570,6 +1570,36 @@
           <t>salinity</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>permeability_unit</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>reservoir_permx</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>overburden_permx</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>oh_perm</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>cb_perm</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>barrier_perm</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1618,6 +1648,16 @@
       <c r="L2" t="n">
         <v>0.032</v>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>mD</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1666,6 +1706,16 @@
       <c r="L3" t="n">
         <v>0.032</v>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>mD</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1705,7 +1755,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GridPolicy and SubsurfaceAssumptions are editable example scenario values and must be reviewed for a real case.</t>
+          <t>GridPolicy and DesignMatrix are editable example scenario values and must be reviewed for a real case.</t>
         </is>
       </c>
     </row>
@@ -1719,7 +1769,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Multiple rows in SubsurfaceAssumptions define a design matrix of scenarios that can be run with --case-name selection.</t>
+          <t>Multiple rows in DesignMatrix define cases that can be run with --case-name selection.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Clarify DesignMatrix permeability scope
Keep open-hole permeability out of per-case sensitivities, document current case-wide cement overrides, and roadmap interval targeting and clearer workbook names.
</commit_message>
<xml_diff>
--- a/test_data/examples/smeaheia/smeaheia_workbook.xlsx
+++ b/test_data/examples/smeaheia/smeaheia_workbook.xlsx
@@ -1506,7 +1506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:Q3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1587,15 +1587,10 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>oh_perm</t>
+          <t>cb_perm</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
-        <is>
-          <t>cb_perm</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
         <is>
           <t>barrier_perm</t>
         </is>
@@ -1657,7 +1652,6 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1715,7 +1709,6 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(gap): target interval permeability overrides
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/test_data/examples/smeaheia/smeaheia_workbook.xlsx
+++ b/test_data/examples/smeaheia/smeaheia_workbook.xlsx
@@ -1506,7 +1506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1595,6 +1595,16 @@
           <t>barrier_perm</t>
         </is>
       </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>cb_perm_interval</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>barrier_perm_interval</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1652,6 +1662,16 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1709,6 +1729,16 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1721,7 +1751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1766,6 +1796,13 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>cb_perm_interval and barrier_perm_interval select a HoleCasings or Plugs name; ALL applies the permeability to every interval of that type.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(gap): add experimental localized casing holes
Support one validated casing hole per scenario with area-conserving positive-X face overrides and resolved metadata. Preserve no-defect output and document pending CIRRUS connectivity verification.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/test_data/examples/smeaheia/smeaheia_workbook.xlsx
+++ b/test_data/examples/smeaheia/smeaheia_workbook.xlsx
@@ -1506,7 +1506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S3"/>
+  <dimension ref="A1:V3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1603,6 +1603,21 @@
       <c r="S1" t="inlineStr">
         <is>
           <t>barrier_perm_interval</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>casing_hole_casing</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>casing_hole_depth_mTVDMSL</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>casing_hole_diameter_m</t>
         </is>
       </c>
     </row>
@@ -1672,6 +1687,9 @@
           <t>ALL</t>
         </is>
       </c>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1739,6 +1757,9 @@
           <t>ALL</t>
         </is>
       </c>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1751,7 +1772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1803,6 +1824,13 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Experimental casing hole: supply casing_hole_casing, casing_hole_depth_mTVDMSL, and casing_hole_diameter_m together, or leave all blank. Placement is fixed on the +X side.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(gap): resolve workbook pressure datums through WellClass
Preserve reservoir depth/pressure anchors when deriving fluid-contact pressure, share resolution across CIRRUS staging and QC, and record resolved inputs. Reject inconsistent pressure pairs and update examples, documentation and regressions.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/test_data/examples/smeaheia/smeaheia_workbook.xlsx
+++ b/test_data/examples/smeaheia/smeaheia_workbook.xlsx
@@ -1506,7 +1506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V3"/>
+  <dimension ref="A1:AB3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1587,37 +1587,67 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>free_fluid_permx</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>free_fluid_poro</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
           <t>cb_perm</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>barrier_perm</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>water_overburden_wall_porv_multiplier</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>reservoir_bottom_porv_multiplier</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>reservoir_wall_porv_multiplier</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
         <is>
           <t>cb_perm_interval</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>barrier_perm_interval</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>casing_hole_casing</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>casing_hole_depth_mTVDMSL</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>casing_hole_diameter_m</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>casing_hole_open</t>
         </is>
       </c>
     </row>
@@ -1677,19 +1707,25 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr"/>
+      <c r="Z2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1747,19 +1783,25 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
       <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1772,7 +1814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1806,28 +1848,35 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>z_fluid_contact and p_fluid_contact define the GAS_WATER datum and WGC depth in CIRRUS.</t>
+          <t>z_fluid_contact alone uses hydrostatic pressure; an explicit p_fluid_contact anchors the contact.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Multiple rows in DesignMatrix define cases that can be run with --case-name selection.</t>
+          <t>z_resrv/p_resrv anchor the CO2 curve; a deeper z_fluid_contact derives its pressure from that curve. Both explicit pairs must agree within 0.01 bar.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>cb_perm_interval and barrier_perm_interval select a HoleCasings or Plugs name; ALL applies the permeability to every interval of that type.</t>
+          <t>Multiple rows in DesignMatrix define cases that can be run with --case-name selection.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Experimental casing hole: supply casing_hole_casing, casing_hole_depth_mTVDMSL, and casing_hole_diameter_m together, or leave all blank. Placement is fixed on the +X side.</t>
+          <t>cb_perm_interval and barrier_perm_interval select a HoleCasings or Plugs name; ALL applies the permeability to every interval of that type.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Experimental casing hole: supply casing_hole_casing, casing_hole_depth_mTVDMSL, and casing_hole_diameter_m together, or leave all blank. Placement is fixed on the +X side. The location also adds FIPHOL reporting (1 inner, 2 outer, 3 rest of the LGR); set casing_hole_open to FALSE for a sealed control with identical reporting.</t>
         </is>
       </c>
     </row>

</xml_diff>